<commit_message>
Update relay expansion and four-channel audio plan
</commit_message>
<xml_diff>
--- a/documentacao/STAYCONTROL_Lista_de_Compras.xlsx
+++ b/documentacao/STAYCONTROL_Lista_de_Compras.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Ra101b146a19f4269"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de compras" sheetId="2" r:id="R1116888c31924e10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes e segurança" sheetId="3" r:id="R158df7b2f80b48a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rd350ef3f867f48db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de compras" sheetId="2" r:id="Raf7b59cb88fc432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes e segurança" sheetId="3" r:id="Rf9fe422d34fd4e04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -413,7 +413,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -424,7 +424,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -435,7 +435,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -769,11 +769,11 @@
       </x:c>
       <x:c r="E6" s="13" t="n">
         <x:f>SUMIFS('Lista de compras'!$L$6:$L$50,'Lista de compras'!$B$6:$B$50,"Quarto")</x:f>
-        <x:v>4189</x:v>
+        <x:v>4284</x:v>
       </x:c>
       <x:c r="F6" s="13" t="n">
         <x:f>SUMIFS('Lista de compras'!$M$6:$M$50,'Lista de compras'!$B$6:$B$50,"Quarto")</x:f>
-        <x:v>7622</x:v>
+        <x:v>7842</x:v>
       </x:c>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="40"/>
@@ -788,7 +788,7 @@
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="39" t="str">
-        <x:v>Relé auxiliar por quarto (0=não; 1=sim)</x:v>
+        <x:v>Banco auxiliar: 2 placas de 16 canais por quarto (0=não; 1=sim)</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="12" t="n">
@@ -799,11 +799,11 @@
       </x:c>
       <x:c r="E7" s="13" t="n">
         <x:f>SUMIFS('Lista de compras'!$L$6:$L$50,'Lista de compras'!$B$6:$B$50,"Auxiliar")</x:f>
-        <x:v>78</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F7" s="13" t="n">
         <x:f>SUMIFS('Lista de compras'!$M$6:$M$50,'Lista de compras'!$B$6:$B$50,"Auxiliar")</x:f>
-        <x:v>162</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="40"/>
@@ -855,11 +855,11 @@
       </x:c>
       <x:c r="E9" s="19" t="n">
         <x:f>SUM('Lista de compras'!$L$6:$L$50)</x:f>
-        <x:v>8897</x:v>
+        <x:v>9106</x:v>
       </x:c>
       <x:c r="F9" s="19" t="n">
         <x:f>SUM('Lista de compras'!$M$6:$M$50)</x:f>
-        <x:v>24234</x:v>
+        <x:v>24532</x:v>
       </x:c>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="40"/>
@@ -881,7 +881,7 @@
       </x:c>
       <x:c r="E10" s="22" t="n">
         <x:f>COUNTBLANK('Lista de compras'!$J$6:$J$50)</x:f>
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="22" t="str">
         <x:v>dimensionar antes da compra</x:v>
@@ -988,10 +988,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B15" s="27" t="str">
-        <x:v>O relé auxiliar é opcional.</x:v>
+        <x:v>Banco auxiliar com 32 canais.</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>A quantidade só entra no orçamento quando C7=1. Ele é destinado a luzes/tomadas extras definidas pelo administrador.</x:v>
+        <x:v>Inclui 2 módulos de 16 relés por quarto; a fonte e a interface de comando precisam ser dimensionadas para a carga real.</x:v>
       </x:c>
       <x:c r="D15" s="27"/>
       <x:c r="E15" s="27"/>
@@ -1012,10 +1012,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B16" s="27" t="str">
-        <x:v>Não ligue compressor de ar-condicionado em relé genérico.</x:v>
+        <x:v>Atualize e valide antes da compra.</x:v>
       </x:c>
       <x:c r="C16" s="27" t="str">
-        <x:v>TV e ar-condicionado são comandados por infravermelho. Cargas de rede exigem contator/proteção dimensionados.</x:v>
+        <x:v>Os 32 auxiliares e o áudio 4 × 50 W exigem interface/firmware, DAC e alimentação dimensionados; os preços sem cotação não entram no total.</x:v>
       </x:c>
       <x:c r="D16" s="27"/>
       <x:c r="E16" s="27"/>
@@ -3583,10 +3583,10 @@
         <x:v>Relés</x:v>
       </x:c>
       <x:c r="D15" s="64" t="str">
-        <x:v>Módulo relé auxiliar de 8 canais</x:v>
+        <x:v>Módulo relé auxiliar de 16 canais (2 placas por quarto)</x:v>
       </x:c>
       <x:c r="E15" s="64" t="str">
-        <x:v>Mesmo padrão do módulo principal; aparece somente no modo administrador</x:v>
+        <x:v>5 V, 16 entradas de comando por placa, optoacoplamento; somente após validar interface e fonte</x:v>
       </x:c>
       <x:c r="F15" s="65" t="n">
         <x:v>0</x:v>
@@ -3595,34 +3595,34 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H15" s="65" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I15" s="66" t="n">
         <x:f>F15+(G15*Resumo!$C$6)+(H15*Resumo!$C$6*Resumo!$C$7)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J15" s="67" t="n">
-        <x:v>43</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="K15" s="67" t="n">
-        <x:v>62</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="L15" s="67" t="n">
         <x:f>IF(OR(I15=0,J15=""),"",I15*J15)</x:f>
-        <x:v>43</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="M15" s="67" t="n">
         <x:f>IF(OR(I15=0,K15=""),"",I15*K15)</x:f>
-        <x:v>62</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="N15" s="68" t="str">
         <x:v>Sob demanda</x:v>
       </x:c>
       <x:c r="O15" s="64" t="str">
-        <x:v>https://www.eletrogate.com/modulo-rele-8-canais-5v</x:v>
+        <x:v>https://vidadesilicio.com.br/produto/modulo-rele-16-canais/</x:v>
       </x:c>
       <x:c r="P15" s="64" t="str">
-        <x:v>Comprar quando os 8 canais principais estiverem ocupados e houver nova luz/tomada.</x:v>
+        <x:v>Configuração: 2 placas × 16 = 32 saídas auxiliares; faixa de referência observada por placa, sem frete. Firmware atual não controla 32 auxiliares.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
@@ -3687,10 +3687,10 @@
         <x:v>Energia</x:v>
       </x:c>
       <x:c r="D17" s="64" t="str">
-        <x:v>Reserva de potência 5 V para expansão</x:v>
+        <x:v>Fonte(s) dedicada(s) para o banco auxiliar</x:v>
       </x:c>
       <x:c r="E17" s="64" t="str">
-        <x:v>Fonte adicional ou fonte maior calculada para 16 relés</x:v>
+        <x:v>Dimensionar para 32 relés auxiliares; verificar corrente de bobina, partidas simultâneas e distribuição por placa</x:v>
       </x:c>
       <x:c r="F17" s="65" t="n">
         <x:v>0</x:v>
@@ -3705,26 +3705,20 @@
         <x:f>F17+(G17*Resumo!$C$6)+(H17*Resumo!$C$6*Resumo!$C$7)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J17" s="67" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="K17" s="67" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="L17" s="67" t="n">
+      <x:c r="J17" s="67"/>
+      <x:c r="K17" s="67"/>
+      <x:c r="L17" s="67" t="str">
         <x:f>IF(OR(I17=0,J17=""),"",I17*J17)</x:f>
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="M17" s="67" t="n">
+      </x:c>
+      <x:c r="M17" s="67" t="str">
         <x:f>IF(OR(I17=0,K17=""),"",I17*K17)</x:f>
-        <x:v>100</x:v>
       </x:c>
       <x:c r="N17" s="68" t="str">
         <x:v>Sob demanda</x:v>
       </x:c>
       <x:c r="O17" s="64" t="str"/>
       <x:c r="P17" s="64" t="str">
-        <x:v>Confirmar consumo das bobinas do módulo escolhido.</x:v>
+        <x:v>Custo não incluído: escolher após confirmar consumo dos módulos e cálculo térmico/elétrico.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="52" customHeight="1">
@@ -4156,10 +4150,10 @@
         <x:v>Áudio</x:v>
       </x:c>
       <x:c r="D26" s="64" t="str">
-        <x:v>Adaptador de áudio USB (DAC)</x:v>
+        <x:v>DAC USB de quatro canais</x:v>
       </x:c>
       <x:c r="E26" s="64" t="str">
-        <x:v>Compatível com Linux/Raspberry Pi OS, saída estéreo</x:v>
+        <x:v>Compatível com Raspberry Pi OS; quatro saídas analógicas independentes para entrada dos amplificadores</x:v>
       </x:c>
       <x:c r="F26" s="65" t="n">
         <x:v>0</x:v>
@@ -4174,26 +4168,20 @@
         <x:f>F26+(G26*Resumo!$C$6)+(H26*Resumo!$C$6*Resumo!$C$7)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J26" s="67" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K26" s="67" t="n">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="L26" s="67" t="n">
+      <x:c r="J26" s="67"/>
+      <x:c r="K26" s="67"/>
+      <x:c r="L26" s="67" t="str">
         <x:f>IF(OR(I26=0,J26=""),"",I26*J26)</x:f>
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="M26" s="67" t="n">
+      </x:c>
+      <x:c r="M26" s="67" t="str">
         <x:f>IF(OR(I26=0,K26=""),"",I26*K26)</x:f>
-        <x:v>160</x:v>
       </x:c>
       <x:c r="N26" s="68" t="str">
         <x:v>Essencial</x:v>
       </x:c>
       <x:c r="O26" s="64" t="str"/>
       <x:c r="P26" s="64" t="str">
-        <x:v>O Raspberry Pi 5 não possui saída analógica P2 integrada.</x:v>
+        <x:v>Não usar o DAC estéreo existente; preço depende do modelo multicanal compatível.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="52" customHeight="1">
@@ -4207,46 +4195,46 @@
         <x:v>Áudio</x:v>
       </x:c>
       <x:c r="D27" s="64" t="str">
-        <x:v>Amplificador estéreo PAM8610 2 × 15 W</x:v>
+        <x:v>Amplificador estéreo Classe D 2 × 50 W (2 unidades)</x:v>
       </x:c>
       <x:c r="E27" s="64" t="str">
-        <x:v>Alimentação 7–15 V, alto-falantes 4–8 Ω</x:v>
+        <x:v>Duas placas estéreo para quatro canais; referência TPA3116D2; saída depende de tensão, impedância, distorção e refrigeração</x:v>
       </x:c>
       <x:c r="F27" s="65" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G27" s="65" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H27" s="65" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I27" s="66" t="n">
         <x:f>F27+(G27*Resumo!$C$6)+(H27*Resumo!$C$6*Resumo!$C$7)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J27" s="67" t="n">
-        <x:v>25</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="K27" s="67" t="n">
-        <x:v>80</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="L27" s="67" t="n">
         <x:f>IF(OR(I27=0,J27=""),"",I27*J27)</x:f>
-        <x:v>25</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="M27" s="67" t="n">
         <x:f>IF(OR(I27=0,K27=""),"",I27*K27)</x:f>
-        <x:v>80</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="N27" s="68" t="str">
         <x:v>Essencial</x:v>
       </x:c>
       <x:c r="O27" s="64" t="str">
-        <x:v>https://www.eletrogate.com/placa-pam-pam8610-15w-15w-2-canais</x:v>
+        <x:v>https://www.recicomp.com.br/produtos/modulo-amplificador-de-audio-tpa3116d2-50w50w-xh-m562/</x:v>
       </x:c>
       <x:c r="P27" s="64" t="str">
-        <x:v>Usar dissipação e caixa ventilada conforme o módulo.</x:v>
+        <x:v>Estimativa unitária provisória; duas placas entregam quatro canais somente após validação de potência RMS, carga e alimentação.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="52" customHeight="1">
@@ -4260,10 +4248,10 @@
         <x:v>Áudio</x:v>
       </x:c>
       <x:c r="D28" s="64" t="str">
-        <x:v>Fonte 12 V / 3 A dedicada ao áudio</x:v>
+        <x:v>Fonte dedicada do amplificador</x:v>
       </x:c>
       <x:c r="E28" s="64" t="str">
-        <x:v>Regulada, baixo ruído, isolada</x:v>
+        <x:v>24 Vcc regulada, alvo inicial 12,5 A (300 W); validar consumo, pico, proteção, ventilação e requisitos dos módulos escolhidos</x:v>
       </x:c>
       <x:c r="F28" s="65" t="n">
         <x:v>0</x:v>
@@ -4278,28 +4266,20 @@
         <x:f>F28+(G28*Resumo!$C$6)+(H28*Resumo!$C$6*Resumo!$C$7)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J28" s="67" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K28" s="67" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="L28" s="67" t="n">
+      <x:c r="J28" s="67"/>
+      <x:c r="K28" s="67"/>
+      <x:c r="L28" s="67" t="str">
         <x:f>IF(OR(I28=0,J28=""),"",I28*J28)</x:f>
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="M28" s="67" t="n">
+      </x:c>
+      <x:c r="M28" s="67" t="str">
         <x:f>IF(OR(I28=0,K28=""),"",I28*K28)</x:f>
-        <x:v>100</x:v>
       </x:c>
       <x:c r="N28" s="68" t="str">
         <x:v>Essencial</x:v>
       </x:c>
-      <x:c r="O28" s="64" t="str">
-        <x:v>https://www.eletrogate.com/placa-pam-pam8610-15w-15w-2-canais</x:v>
-      </x:c>
+      <x:c r="O28" s="64"/>
       <x:c r="P28" s="64" t="str">
-        <x:v>Separar da fita RGB reduz ruídos audíveis.</x:v>
+        <x:v>Preço não incluído até fechar o amplificador e a carga. Dimensionamento final por profissional; fonte isolada e protegida.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="52" customHeight="1">
@@ -4313,23 +4293,23 @@
         <x:v>Áudio</x:v>
       </x:c>
       <x:c r="D29" s="64" t="str">
-        <x:v>Alto-falante 15 W, 4–8 Ω</x:v>
+        <x:v>Alto-falante de 50 W RMS, 4–8 Ω</x:v>
       </x:c>
       <x:c r="E29" s="64" t="str">
-        <x:v>Full range, próprio para embutir; par estéreo</x:v>
+        <x:v>Full range compatível com a impedância e potência real de cada canal; quatro unidades</x:v>
       </x:c>
       <x:c r="F29" s="65" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G29" s="65" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H29" s="65" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I29" s="66" t="n">
         <x:f>F29+(G29*Resumo!$C$6)+(H29*Resumo!$C$6*Resumo!$C$7)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J29" s="67" t="n">
         <x:v>50</x:v>
@@ -4339,11 +4319,11 @@
       </x:c>
       <x:c r="L29" s="67" t="n">
         <x:f>IF(OR(I29=0,J29=""),"",I29*J29)</x:f>
-        <x:v>100</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="M29" s="67" t="n">
         <x:f>IF(OR(I29=0,K29=""),"",I29*K29)</x:f>
-        <x:v>320</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="N29" s="68" t="str">
         <x:v>Essencial</x:v>
@@ -4401,7 +4381,7 @@
       </x:c>
       <x:c r="O30" s="64" t="str"/>
       <x:c r="P30" s="64" t="str">
-        <x:v>Manter afastado dos cabos de rede elétrica.</x:v>
+        <x:v>Dimensionar bitola e comprimento para quatro canais; separar sinal de linha da saída amplificada.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="52" customHeight="1">

</xml_diff>